<commit_message>
feat(prospects): clickable urls/emails in xlsx; rebuild zip + download page
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prospects/Target-Companies.xlsx
+++ b/prospects/Target-Companies.xlsx
@@ -2348,7 +2348,7 @@
       <c r="I2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="K2" s="4" t="s">
@@ -2548,7 +2548,7 @@
       <c r="I5" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="6" t="s">
         <v>87</v>
       </c>
       <c r="K5" s="4" t="s">
@@ -2616,7 +2616,7 @@
       <c r="I6" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="6" t="s">
         <v>104</v>
       </c>
       <c r="K6" s="4" t="s">
@@ -3014,7 +3014,7 @@
       <c r="I12" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="6" t="s">
         <v>191</v>
       </c>
       <c r="K12" s="4" t="s">
@@ -3148,7 +3148,7 @@
       <c r="I14" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="6" t="s">
         <v>224</v>
       </c>
       <c r="K14" s="4" t="s">
@@ -3284,7 +3284,7 @@
       <c r="I16" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="6" t="s">
         <v>253</v>
       </c>
       <c r="K16" s="4" t="s">
@@ -3352,7 +3352,7 @@
       <c r="I17" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="J17" s="6" t="s">
         <v>268</v>
       </c>
       <c r="K17" s="4" t="s">
@@ -3420,7 +3420,7 @@
       <c r="I18" s="4" t="s">
         <v>283</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="J18" s="6" t="s">
         <v>284</v>
       </c>
       <c r="K18" s="4" t="s">
@@ -3612,7 +3612,7 @@
       <c r="I21" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="J21" s="4" t="s">
+      <c r="J21" s="6" t="s">
         <v>324</v>
       </c>
       <c r="K21" s="4" t="s">
@@ -3680,7 +3680,7 @@
       <c r="I22" s="4" t="s">
         <v>338</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="J22" s="6" t="s">
         <v>339</v>
       </c>
       <c r="K22" s="4" t="s">
@@ -3946,7 +3946,7 @@
       <c r="I26" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="J26" s="4" t="s">
+      <c r="J26" s="6" t="s">
         <v>395</v>
       </c>
       <c r="K26" s="4" t="s">
@@ -4146,7 +4146,7 @@
       <c r="I29" s="4" t="s">
         <v>439</v>
       </c>
-      <c r="J29" s="4" t="s">
+      <c r="J29" s="6" t="s">
         <v>440</v>
       </c>
       <c r="K29" s="4" t="s">
@@ -4190,25 +4190,37 @@
   <autoFilter ref="A1:V29"/>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1"/>
-    <hyperlink ref="F3" r:id="rId2"/>
-    <hyperlink ref="F4" r:id="rId3"/>
-    <hyperlink ref="F5" r:id="rId4"/>
-    <hyperlink ref="F6" r:id="rId5"/>
-    <hyperlink ref="F7" r:id="rId6"/>
-    <hyperlink ref="F9" r:id="rId7"/>
-    <hyperlink ref="F12" r:id="rId8"/>
-    <hyperlink ref="F14" r:id="rId9"/>
-    <hyperlink ref="F15" r:id="rId10"/>
-    <hyperlink ref="F16" r:id="rId11"/>
-    <hyperlink ref="F17" r:id="rId12"/>
-    <hyperlink ref="F18" r:id="rId13"/>
-    <hyperlink ref="F21" r:id="rId14"/>
-    <hyperlink ref="F22" r:id="rId15"/>
-    <hyperlink ref="F24" r:id="rId16"/>
-    <hyperlink ref="F25" r:id="rId17"/>
-    <hyperlink ref="F26" r:id="rId18"/>
-    <hyperlink ref="F28" r:id="rId19"/>
-    <hyperlink ref="F29" r:id="rId20"/>
+    <hyperlink ref="J2" r:id="rId2"/>
+    <hyperlink ref="F3" r:id="rId3"/>
+    <hyperlink ref="F4" r:id="rId4"/>
+    <hyperlink ref="F5" r:id="rId5"/>
+    <hyperlink ref="J5" r:id="rId6"/>
+    <hyperlink ref="F6" r:id="rId7"/>
+    <hyperlink ref="J6" r:id="rId8"/>
+    <hyperlink ref="F7" r:id="rId9"/>
+    <hyperlink ref="F9" r:id="rId10"/>
+    <hyperlink ref="F12" r:id="rId11"/>
+    <hyperlink ref="J12" r:id="rId12"/>
+    <hyperlink ref="F14" r:id="rId13"/>
+    <hyperlink ref="J14" r:id="rId14"/>
+    <hyperlink ref="F15" r:id="rId15"/>
+    <hyperlink ref="F16" r:id="rId16"/>
+    <hyperlink ref="J16" r:id="rId17"/>
+    <hyperlink ref="F17" r:id="rId18"/>
+    <hyperlink ref="J17" r:id="rId19"/>
+    <hyperlink ref="F18" r:id="rId20"/>
+    <hyperlink ref="J18" r:id="rId21"/>
+    <hyperlink ref="F21" r:id="rId22"/>
+    <hyperlink ref="J21" r:id="rId23"/>
+    <hyperlink ref="F22" r:id="rId24"/>
+    <hyperlink ref="J22" r:id="rId25"/>
+    <hyperlink ref="F24" r:id="rId26"/>
+    <hyperlink ref="F25" r:id="rId27"/>
+    <hyperlink ref="F26" r:id="rId28"/>
+    <hyperlink ref="J26" r:id="rId29"/>
+    <hyperlink ref="F28" r:id="rId30"/>
+    <hyperlink ref="F29" r:id="rId31"/>
+    <hyperlink ref="J29" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>

</xml_diff>

<commit_message>
feat: fill social channels for 17 prospects; add 3 half-day walkthrough interview guides (Yangtze S/A)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prospects/Target-Companies.xlsx
+++ b/prospects/Target-Companies.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="941">
   <si>
     <t>长三角 · 珠三角 重点客户（按初筛分排序）</t>
   </si>
@@ -249,7 +249,7 @@
     <t>15711700118（政采投标专线）· 15710701718（工厂报价/方案）· 16616656119（外贸）</t>
   </si>
   <si>
-    <t>品牌公众号与视频号（VOU+卫域）—— 本轮未采到具体账号，可电话索取</t>
+    <t>品牌名「VOU+卫域」可在微信搜一搜直接找公众号/视频号；官网同时挂 Wechat/WhatsApp：15710701718（询盘即达）</t>
   </si>
   <si>
     <t>政采投标专线 15711700118（对口项目）；工厂报价/方案 15710701718；邮箱 sampu@vouplus.com 备用</t>
@@ -273,7 +273,7 @@
     <t>021-64500738 · 17721000960</t>
   </si>
   <si>
-    <t>（待补）—— 官网无社媒入口</t>
+    <t>官网 News/案例栏目持续更新（乐高、Coach、祖·玛珑、KOSE-Albion、DR 等案例）；微信同号 17721000960；无公众号/抖音入口</t>
   </si>
   <si>
     <t>021-64500738 总机 + 17721000960；Business@zg-huayue.com 发「快闪店到店时间」案例</t>
@@ -309,10 +309,10 @@
     <t>门业</t>
   </si>
   <si>
-    <t>维持 A —— 官网未找到，改走永康国际门业博览会现场核实</t>
-  </si>
-  <si>
-    <t>（待补）—— 官网未找到，改走永康国际门业博览会现场</t>
+    <t>维持 A —— 无官网；2026-06 企业专访证实为中外合资（吉尔吉斯斯坦+浙江德福隆）、600+ 经销商 / 200+ 专卖店、双品牌「德艺 / 贵府」，改走经销商体系与永康门博会</t>
+  </si>
+  <si>
+    <t>无独立官网亦无社媒入口 → 线上替代：微信搜一搜「德艺门业」「德艺贵府」（双品牌），或走 600+ 经销商网络与永康国际门业博览会</t>
   </si>
   <si>
     <t>官网未找到 → 走永康国际门业博览会现场（展位谈 10 分钟）或门都门业协会名录</t>
@@ -369,7 +369,7 @@
     <t>021-57406543（营销中心）· 021-57401515（总机）</t>
   </si>
   <si>
-    <t>（待补）—— 新三板挂牌企业，官网以招商与案例为主</t>
+    <t>（待补）—— 挂牌公司官网 hooyigroup.com 以案例与招商为主，微信入口需官网在线留言索取</t>
   </si>
   <si>
     <t>营销中心 021-57406543 / 总机 021-57401515；yxtz@hooyigroup.com；挂牌公司有专职对接人，直接问「信息化负责人」</t>
@@ -411,7 +411,7 @@
     <t>137-0297-9732（渠道）· 17052431054（工厂）</t>
   </si>
   <si>
-    <t>（待补）—— 品牌站 fsclover.com</t>
+    <t>官网品牌站 fsclover.com + 老站 gdclover.com（英文）；「OEM 代加工」页为 B 端入口；无公众号/抖音入口</t>
   </si>
   <si>
     <t>137-0297-9732 / 17052431054；595565222@qq.com；开场就说「只补车间那一段，不动你现有系统」</t>
@@ -429,7 +429,7 @@
     <t>15813445274</t>
   </si>
   <si>
-    <t>（待补）—— 无独立官网，走厂家直销电话</t>
+    <t>（待补）—— 无独立官网；线上替代：厂家直销微信 13924888502 + 邮箱 2385922529@qq.com，先确认与「伍发门窗」的主体关系</t>
   </si>
   <si>
     <t>厂家直销 13924888502；2385922529@qq.com；先确认 weps168.com 页面同时出现「伍发门窗」的主体关系</t>
@@ -489,7 +489,7 @@
     <t>400-112-0007（集团）· 0579-89083098</t>
   </si>
   <si>
-    <t>（待补）—— 集团官网 kkdgroup.com 有「视频中心」栏目，可作内容触点</t>
+    <t>集团官网 kkdgroup.com 设「视频中心」栏目 + 招商加盟在线报名（B 端入口）；公众号可微信搜「金凯德」</t>
   </si>
   <si>
     <t>400-112-0007（集团）转安防事业部；0579-89083098；只谈武义单一厂区，别谈集团</t>
@@ -543,7 +543,7 @@
     <t>021-59556615 · 传真 021-59556342</t>
   </si>
   <si>
-    <t>（待补）—— 无官网</t>
+    <t>无官网亦无社媒入口 → 线上替代：021-59556615 电话直连（传真 021-59556342）</t>
   </si>
   <si>
     <t>021-59556615（传真 021-59556342）；无官网，先电话确认现名与厂址（嘉定区新建一路 2305 号）</t>
@@ -588,7 +588,7 @@
     <t>0571-58982959（行政/客服）· 0571-58982988（销售）· 传真 0571-58837981</t>
   </si>
   <si>
-    <t>（待补）—— 上市公司，节奏按月算</t>
+    <t>（待补）—— 上市公司：上交所/公司公告是权威信息源（比社媒可靠）；官网 hdnew.cn 可查投资者关系入口</t>
   </si>
   <si>
     <t>销售 0571-58982988 / 行政 0571-58982959；hdnew@hdnew.cn；走投关/信息化双通道，节奏按月算</t>
@@ -657,7 +657,7 @@
     <t>400 电话（工商页掩码，官网查询）</t>
   </si>
   <si>
-    <t>（待补）—— 集团官网 onlead.com.cn 在线留言</t>
+    <t>官网 onlead.com.cn 在线留言入口；400 电话以官网公示为准；集团化企业走「集团信息化」对口</t>
   </si>
   <si>
     <t>官网 www.onlead.com.cn 在线留言 → 转集团信息化；400 电话以官网公示为准</t>
@@ -744,7 +744,7 @@
     <t>+86 755 21614789（深圳办公室，中国区）· +60 7 7069901（马来西亚）</t>
   </si>
   <si>
-    <t>（待补）—— 走集团投关/招商通道</t>
+    <t>（待补）—— 走集团通道（投关/招商），官网 cimc.com；对口邮箱 modulardc@cimc.com</t>
   </si>
   <si>
     <t>深圳办公室 +86 755 21614789；modulardc@cimc.com；只谈江门工厂的模块齐套场景</t>
@@ -1008,13 +1008,13 @@
     <t>浙江</t>
   </si>
   <si>
-    <t>未找到官网（多轮检索未命中企业主体页）</t>
-  </si>
-  <si>
-    <t>（待核实：防火门/入户门方向）</t>
-  </si>
-  <si>
-    <t>✗ 未验证：原线索来自门业榜单与推广页；建议改走【永康国际门业博览会】现场核实，或从门都门业协会名录取准确全称与信用代码后再联系</t>
+    <t>无独立官网（多轮检索未命中）；公开报道可查</t>
+  </si>
+  <si>
+    <t>双品牌「德艺 / 贵府」：铸铝门、铜门、高端防盗门、防火门、钢质进户门；自述「通轴技术」为核心卖点</t>
+  </si>
+  <si>
+    <t>△ 部分（有实质补充）：官网仍未找到，但 2026-06 中华网企业专访披露——中外合资（吉尔吉斯斯坦德氏贸易 + 浙江德福隆电子材料联合设立）、深耕高端门业十余年、600+ 经销商、200+ 专卖店、产品出口东南亚/中东/欧美；获国家高新技术企业、「浙江制造」品字标、浙江省创新型中小企业。规模与渠道比原判断大得多，维持 A 级，但触达走经销商体系而非官网</t>
   </si>
   <si>
     <t>浙江金华永康（待核实）</t>
@@ -1032,7 +1032,7 @@
     <t>一樘门完整档案（钢板批号→消防验收）+投标台账导出</t>
   </si>
   <si>
-    <t>检索未命中 · 核实日 2026-09-11</t>
+    <t>中华网企业专访（2026-06-03）· 永康门博会与协会名录（建议） · 核实日 2026-09-12</t>
   </si>
   <si>
     <t>https://www.hooyigroup.com</t>
@@ -1974,7 +1974,7 @@
     <t>山东省滨州市博兴县店子工业园区（邮编 256508）</t>
   </si>
   <si>
-    <t>（待补）</t>
+    <t>官网有「企业视频」栏目 + 云展网电子画册（yunzhan365.com/read/osyy）；线上替代触点：顺企网/黄页店铺 + 官网在线留言（400-0543-999）——首页/页脚无公众号入口</t>
   </si>
   <si>
     <t>全国线 400-0543-999；国际贸易部 0543-2969077/78/79（外贸线索从这条进）；人力 0543-2969042 问系统岗是否在招</t>
@@ -2118,6 +2118,9 @@
     <t>四川省成都市崇州经济开发区晨曦大道南段 429 号</t>
   </si>
   <si>
+    <t>官网底部「官方微信」二维码（扫码关注）+ 「视频宣传」栏目；另有在线报修/派单/定位签到入口（说明已有服务端系统）</t>
+  </si>
+  <si>
     <t>400-880-7215 → 转信息/生产；028-85750608 总部；邮箱 cdhuihong@163.com</t>
   </si>
   <si>
@@ -2160,6 +2163,9 @@
     <t>山东省滨州市博兴县兴福镇福旺白铁市场</t>
   </si>
   <si>
+    <t>（待补）—— 官网口径停留在 2013 年；线上替代：0543-2760067 电话 + jintailigangtie@163.com，先核实现状</t>
+  </si>
+  <si>
     <t>0543-2760067 / 0543-2760019；jintailigangtie@163.com；先核实 2013 年之后产线有无增减</t>
   </si>
   <si>
@@ -2244,7 +2250,7 @@
     <t>天津市西青区精武镇南河工业园民兴路 8 号</t>
   </si>
   <si>
-    <t>（待补）—— 作为标杆案例素材，暂不投入</t>
+    <t>（待补）—— 线上替代：400-630-8518（24 小时）+ xinyucaiban@126.com；作为标杆案例素材，暂不投入</t>
   </si>
   <si>
     <t>400-630-8518（24h）；xinyucaiban@126.com；作为标杆案例素材，不作为试点客户</t>
@@ -2295,6 +2301,9 @@
     <t>河北省沧州市河间市边边工业区（注册主体名是任丘，厂址在河间）</t>
   </si>
   <si>
+    <t>（待补）—— 无官网；线上替代：总机 13513493191 + z17121055555@163.com；工程案例（医院/法院/万达）可作谈资</t>
+  </si>
+  <si>
     <t>总机 13513493191 / 邮箱 z17121055555@163.com；地址在河间市边边工业区（不是任丘市区）；先问「被动门这条线跑起来了没」</t>
   </si>
   <si>
@@ -2338,6 +2347,9 @@
   </si>
   <si>
     <t>沈阳市浑南区文溯街 17-48 号</t>
+  </si>
+  <si>
+    <t>（待补）—— 仅有 B2B 页面；线上替代：024-24770099（备用 15804006911）</t>
   </si>
   <si>
     <t>024-24770099（备用 15804006911）；先核实是否仍做防火门工程与年产规模</t>
@@ -5228,7 +5240,7 @@
         <v>268</v>
       </c>
       <c r="X8" s="4" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="104" customHeight="1">
@@ -7539,16 +7551,16 @@
         <v>697</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>650</v>
+        <v>698</v>
       </c>
       <c r="N40" s="5" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="O40" s="5" t="s">
         <v>126</v>
       </c>
       <c r="P40" s="5" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="Q40" s="4" t="s">
         <v>17</v>
@@ -7557,16 +7569,16 @@
         <v>112</v>
       </c>
       <c r="S40" s="5" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="T40" s="5" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="U40" s="5" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="V40" s="5" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="W40" s="4" t="s">
         <v>268</v>
@@ -7580,13 +7592,13 @@
         <v>358</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C41" s="18" t="s">
         <v>606</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>608</v>
@@ -7595,34 +7607,34 @@
         <v>609</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="J41" s="5" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="K41" s="13" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>650</v>
+        <v>713</v>
       </c>
       <c r="N41" s="5" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="O41" s="5" t="s">
         <v>184</v>
       </c>
       <c r="P41" s="5" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="Q41" s="4" t="s">
         <v>185</v>
@@ -7631,16 +7643,16 @@
         <v>147</v>
       </c>
       <c r="S41" s="5" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="T41" s="5" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="U41" s="5" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="V41" s="5" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="W41" s="4" t="s">
         <v>268</v>
@@ -7654,43 +7666,43 @@
         <v>358</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>608</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="H42" s="5"/>
       <c r="I42" s="5" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="J42" s="5"/>
       <c r="K42" s="5"/>
       <c r="L42" s="5" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="M42" s="5" t="s">
         <v>193</v>
       </c>
       <c r="N42" s="5" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="O42" s="5" t="s">
         <v>184</v>
       </c>
       <c r="P42" s="5" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="Q42" s="4" t="s">
         <v>185</v>
@@ -7699,13 +7711,13 @@
         <v>147</v>
       </c>
       <c r="S42" s="5" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="T42" s="5" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="U42" s="5" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="V42" s="5" t="s">
         <v>428</v>
@@ -7722,49 +7734,49 @@
         <v>358</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C43" s="18" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="K43" s="13" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="M43" s="5" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="N43" s="5" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="O43" s="5" t="s">
         <v>184</v>
       </c>
       <c r="P43" s="5" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="Q43" s="4" t="s">
         <v>185</v>
@@ -7773,16 +7785,16 @@
         <v>165</v>
       </c>
       <c r="S43" s="5" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="T43" s="5" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="U43" s="5" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="V43" s="5" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="W43" s="4" t="s">
         <v>268</v>
@@ -7796,49 +7808,49 @@
         <v>358</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>626</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="K44" s="13" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="M44" s="5" t="s">
-        <v>650</v>
+        <v>759</v>
       </c>
       <c r="N44" s="5" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="O44" s="5" t="s">
         <v>94</v>
       </c>
       <c r="P44" s="5" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="Q44" s="4" t="s">
         <v>17</v>
@@ -7847,13 +7859,13 @@
         <v>203</v>
       </c>
       <c r="S44" s="5" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="T44" s="5" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="U44" s="5" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="V44" s="5" t="s">
         <v>500</v>
@@ -7870,47 +7882,47 @@
         <v>358</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="C45" s="18" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="K45" s="5"/>
       <c r="L45" s="5" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="M45" s="5" t="s">
-        <v>650</v>
+        <v>775</v>
       </c>
       <c r="N45" s="5" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="O45" s="5" t="s">
         <v>94</v>
       </c>
       <c r="P45" s="5" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="Q45" s="4" t="s">
         <v>17</v>
@@ -7919,16 +7931,16 @@
         <v>203</v>
       </c>
       <c r="S45" s="5" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="T45" s="5" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="U45" s="5" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="V45" s="5" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="W45" s="4" t="s">
         <v>389</v>
@@ -8014,70 +8026,70 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="19" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="20" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="20" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="20" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="19" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -8088,13 +8100,13 @@
         <v>244</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1">
@@ -8108,10 +8120,10 @@
         <v>36</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1">
@@ -8125,10 +8137,10 @@
         <v>52</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1">
@@ -8142,10 +8154,10 @@
         <v>52</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1">
@@ -8159,10 +8171,10 @@
         <v>80</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1">
@@ -8176,10 +8188,10 @@
         <v>112</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1">
@@ -8193,10 +8205,10 @@
         <v>147</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1">
@@ -8210,10 +8222,10 @@
         <v>165</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1">
@@ -8227,10 +8239,10 @@
         <v>229</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1">
@@ -8244,10 +8256,10 @@
         <v>36</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1">
@@ -8261,10 +8273,10 @@
         <v>52</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1">
@@ -8278,10 +8290,10 @@
         <v>80</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1">
@@ -8295,10 +8307,10 @@
         <v>112</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1">
@@ -8312,10 +8324,10 @@
         <v>147</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1">
@@ -8329,10 +8341,10 @@
         <v>165</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1">
@@ -8346,10 +8358,10 @@
         <v>203</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1">
@@ -8363,79 +8375,79 @@
         <v>222</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="19" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="3" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="30" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="30" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="30" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="30" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>838</v>
+        <v>842</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="30" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="30" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="30" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="30" customHeight="1">
@@ -8443,68 +8455,68 @@
         <v>164</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="30" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="30" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="30" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="30" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="30" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="19" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="46" customHeight="1">
       <c r="A48" s="3" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="60" customHeight="1">
       <c r="A50" s="3" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
     </row>
   </sheetData>
@@ -8524,267 +8536,267 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="19" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="30" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="30" customHeight="1">
       <c r="A6" s="3" t="s">
+        <v>872</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>868</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>864</v>
-      </c>
       <c r="C6" s="2" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="30" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="30" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="30" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="30" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="19" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="30" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="30" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="30" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="30" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="30" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="30" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="19" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="30" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="2" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="2" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="30" customHeight="1">
       <c r="A24" s="3" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="2" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="2" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="19" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="30" customHeight="1">
       <c r="A28" s="3" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="2" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="30" customHeight="1">
       <c r="A29" s="3" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="2" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="19" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="30" customHeight="1">
       <c r="A32" s="3" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="2" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="30" customHeight="1">
       <c r="A33" s="3" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="2" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="30" customHeight="1">
       <c r="A34" s="3" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="2" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
     </row>
   </sheetData>
@@ -8803,36 +8815,36 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="44" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="44" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="44" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="19" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="58" customHeight="1">
@@ -8840,7 +8852,7 @@
         <v>24</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="58" customHeight="1">
@@ -8848,65 +8860,65 @@
         <v>14</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="58" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="19" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="60" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="60" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="60" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="60" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="19" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="78" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
     </row>
   </sheetData>

</xml_diff>